<commit_message>
submit AI audit log slot 4
</commit_message>
<xml_diff>
--- a/AI Audit Log_LeDinhThuyDuong.xlsx
+++ b/AI Audit Log_LeDinhThuyDuong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\ai-audit-log-DuongLDT2005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0ADECA5-9CF9-4C98-B604-994343752E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C32A6A1-7F7E-435B-B2E5-727DD8ED15E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -94,6 +94,23 @@
   <si>
     <t>Phản hồi: AI giải thích các thành phần của Use Case Description trong Use Case Model gồm: Use Case Name, Summary, Dependency, Actors, Preconditions, Main Sequence, Alternative Sequences, Nonfunctional Requirements, Postconditions và Outstanding Questions; đồng thời giải thích vai trò của từng mục và đưa ví dụ áp dụng.
 Kiểm chứng: Tôi đối chiếu với nội dung tài liệu Software Modeling &amp; Design để xác nhận các thành phần của Use Case Description.</t>
+  </si>
+  <si>
+    <t>“Monitor Sales Dashboard có nên đổi thành use case thống kê không?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích Monitor mang nghĩa giám sát, không phù hợp nếu hệ thống chỉ hiển thị thống kê; đề xuất View Sales Statistics hoặc View Sales Analytics.
+Quyết định: Tôi đổi use case để phản ánh đúng chức năng hệ thống thay vì dùng thuật ngữ chưa chính xác.</t>
+  </si>
+  <si>
+    <t>“Manager có được quyền View Sales Statistics không?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích Manager cần quyền xem thống kê để quản lý doanh thu, thực đơn và hiệu suất bán hàng.
+Quyết định: Tôi giữ quyền View Sales Statistics cho Manager và Admin.</t>
+  </si>
+  <si>
+    <t>Slot 4</t>
   </si>
 </sst>
 </file>
@@ -511,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBDDC7E-59F2-4CBB-B3D2-F6FB78F9E873}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.9375" customWidth="1"/>
@@ -619,6 +636,34 @@
         <v>16</v>
       </c>
     </row>
+    <row r="8" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
submit AI audit log slot 5
</commit_message>
<xml_diff>
--- a/AI Audit Log_LeDinhThuyDuong.xlsx
+++ b/AI Audit Log_LeDinhThuyDuong.xlsx
@@ -8,15 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\ai-audit-log-DuongLDT2005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C32A6A1-7F7E-435B-B2E5-727DD8ED15E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C03F22A1-5FEF-40B7-A4DC-1DE40F852BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
-    <sheet name="Week 3" sheetId="2" r:id="rId2"/>
-    <sheet name="Assignment 2" sheetId="3" r:id="rId3"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Week 3" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="30">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -111,6 +109,30 @@
   </si>
   <si>
     <t>Slot 4</t>
+  </si>
+  <si>
+    <t>Slot 5</t>
+  </si>
+  <si>
+    <t>“Tổng hợp outline kiến thức chương 7 Static Modeling.”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI tổng hợp các nội dung chính của chương gồm: association, aggregation, composition, inheritance, constraints, entity classes, system context, stereotypes. Kiểm chứng: Tôi đối chiếu với cấu trúc chương trong sách để xác nhận các mục lớn được bao phủ đầy đủ.</t>
+  </si>
+  <si>
+    <t>“Phân biệt composition và aggregation.”</t>
+  </si>
+  <si>
+    <t>“Tạo bảng phân biệt các quan hệ trong class diagram và hiệu số.”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI lập bảng so sánh các loại quan hệ UML, gồm association, aggregation, composition, inheritance,… và mô tả mức độ liên kết. Quyết định: Tôi nhận thấy có bổ sung quan hệ ngoài phạm vi chương nên cần tinh chỉnh theo tài liệu học.</t>
+  </si>
+  <si>
+    <t>“Chỉ liệt kê những quan hệ có trong sách thôi.”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giới hạn lại còn association, aggregation, composition và generalization/inheritance; đồng thời nêu các biến thể multiplicity và association types. Kiểm chứng: Tôi dùng kết quả này làm chuẩn khi ôn tập theo đúng nội dung sách thay vì UML mở rộng.</t>
   </si>
 </sst>
 </file>
@@ -596,7 +618,7 @@
     </row>
     <row r="5" spans="1:5" ht="54" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>4</v>
@@ -610,7 +632,7 @@
     </row>
     <row r="6" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>4</v>
@@ -624,7 +646,7 @@
     </row>
     <row r="7" spans="1:5" ht="108" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>4</v>
@@ -638,7 +660,7 @@
     </row>
     <row r="8" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>21</v>
@@ -652,7 +674,7 @@
     </row>
     <row r="9" spans="1:5" ht="54" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>21</v>
@@ -671,28 +693,88 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E3EFE9-6FFB-49CC-BE69-0C0E36C6253E}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEBA1D7F-8E89-493A-8831-E6BA63B86434}">
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="20.9375" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="3" width="28.5" customWidth="1"/>
+    <col min="4" max="4" width="54.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="13.9" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
submit AI audit log week 3
</commit_message>
<xml_diff>
--- a/AI Audit Log_LeDinhThuyDuong.xlsx
+++ b/AI Audit Log_LeDinhThuyDuong.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\ai-audit-log-DuongLDT2005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C03F22A1-5FEF-40B7-A4DC-1DE40F852BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C91DED5-DF6A-4B30-A1B9-B0AAF9643BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="46">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -133,6 +133,54 @@
   </si>
   <si>
     <t>Phản hồi: AI giới hạn lại còn association, aggregation, composition và generalization/inheritance; đồng thời nêu các biến thể multiplicity và association types. Kiểm chứng: Tôi dùng kết quả này làm chuẩn khi ôn tập theo đúng nội dung sách thay vì UML mở rộng.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI xác định các entity classes từ yêu cầu nghiệp vụ (Customer, Booking, Vehicle, Payment, Staff, ...), xây dựng các quan hệ association, multiplicity và inheritance phù hợp rồi sinh mã PlantUML. Quyết định: Tôi sử dụng sơ đồ này làm bản nháp thiết kế trước khi tự kiểm tra lại theo nguyên tắc phân tích miền nghiệp vụ.</t>
+  </si>
+  <si>
+    <t>"Tại sao service với repo thì là use?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích dependency («use») biểu diễn sự phụ thuộc tạm thời giữa các lớp kỹ thuật. Quyết định: Tôi áp dụng dependency thay vì association cho Service và Repository trong design class diagram.</t>
+  </si>
+  <si>
+    <t>"Dựa vào đề AutoGo thiết kế hệ thống và generate class diagram PlantUML."</t>
+  </si>
+  <si>
+    <t>"Có thể gộp Authentication và User Management vào một Class Diagram không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích có thể gộp khi hai chức năng liên quan chặt chẽ thông qua User Entity. Quyết định: Thiết kế diagram chung cho Auth &amp; User Management.</t>
+  </si>
+  <si>
+    <t>"deletedBy trong User có relationship gì không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI xác định đây là self-association giữa User và User. Quyết định: Thêm quan hệ User → User với vai trò deletes.</t>
+  </si>
+  <si>
+    <t>"Các feature có kế thừa interface generic hay abstract class không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích JavaScript không có interface và abstract class thực sự như Java/C#, nhưng UML vẫn có thể biểu diễn. Quyết định: Không sử dụng generic interface trong dự án NodeJS hiện tại.</t>
+  </si>
+  <si>
+    <t>"Shared class có nên vẽ trong diagram không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích sự khác nhau giữa Feature Diagram và Architecture Diagram. Quyết định: Chỉ vẽ shared classes thực sự được sử dụng trong feature đó.</t>
+  </si>
+  <si>
+    <t>"Dependency có cần bỏ trong &lt;&lt;&gt;&gt; không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích stereotype &lt;&lt;dependency&gt;&gt; không cần thiết vì mũi tên ..&gt; đã biểu diễn Dependency. Quyết định: Dùng nhãn như uses, accesses, manages thay cho stereotype.</t>
+  </si>
+  <si>
+    <t>"Gen Class Diagram riêng cho User Management."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI tách User Management khỏi Authentication thành diagram độc lập. Quyết định: Áp dụng phương pháp vẽ diagram theo từng feature/module.</t>
   </si>
 </sst>
 </file>
@@ -694,7 +742,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEBA1D7F-8E89-493A-8831-E6BA63B86434}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.9375" customWidth="1"/>
@@ -774,7 +822,120 @@
         <v>29</v>
       </c>
     </row>
+    <row r="6" spans="1:5" ht="81" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="27" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
submit AI audit log slot 7
</commit_message>
<xml_diff>
--- a/AI Audit Log_LeDinhThuyDuong.xlsx
+++ b/AI Audit Log_LeDinhThuyDuong.xlsx
@@ -1,41 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\ai-audit-log-DuongLDT2005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C91DED5-DF6A-4B30-A1B9-B0AAF9643BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7BFA9A-6E47-48D0-B2F0-477A5BE5EC38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
     <sheet name="Week 3" sheetId="5" r:id="rId2"/>
+    <sheet name="Week 4" sheetId="6" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="59">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -181,6 +173,45 @@
   </si>
   <si>
     <t>Phản hồi: AI tách User Management khỏi Authentication thành diagram độc lập. Quyết định: Áp dụng phương pháp vẽ diagram theo từng feature/module.</t>
+  </si>
+  <si>
+    <t>"Phân tích class diagram Authentication Feature."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích vai trò của Controller, Service, Repository, Entity, Utility và các quan hệ dependency/association trong diagram. Quyết định: Tôi đối chiếu với kiến trúc ExpressJS + Mongoose của dự án để xác nhận các lớp và trách nhiệm phù hợp với implementation thực tế.</t>
+  </si>
+  <si>
+    <t>"Đánh giá các relationship trong Authentication Class Diagram."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích dependency, association, multiplicity giữa User, RefreshToken, PasswordResetToken và Repository. Quyết định: Tôi rà soát lại các quan hệ để bảo đảm đúng ý nghĩa nghiệp vụ và thống nhất cách biểu diễn UML.</t>
+  </si>
+  <si>
+    <t>"Cải thiện Authentication Class Diagram và sinh lại PlantUML."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất loại bỏ các JWT methods khỏi User entity, bổ sung stereotype và điều chỉnh dependency giữa các lớp. Quyết định: Tôi cập nhật diagram theo hướng tách biệt rõ Authentication concern khỏi Entity.</t>
+  </si>
+  <si>
+    <t>"Phân tích User Management Class Diagram."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đánh giá trách nhiệm của UserController, UserService, UserRepository, User entity và chỉ ra các thành phần có thể không thuộc phạm vi User Management. Quyết định: Tôi điều chỉnh lại phạm vi chức năng của feature theo đúng use case quản lý người dùng.</t>
+  </si>
+  <si>
+    <t>"User entity có nên chứa generateAccessToken() và generateRefreshToken() không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích việc tạo JWT thuộc Authentication concern và nên đặt ở Service hoặc Utility thay vì Entity. Quyết định: Tôi loại bỏ các JWT methods khỏi User entity để tăng tính tách biệt trách nhiệm</t>
+  </si>
+  <si>
+    <t>"Sinh lại PlantUML cho User Management Feature sau khi cải thiện."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI tạo lại PlantUML với stereotype, dependency và association đã được chỉnh sửa. Quyết định: Tôi sử dụng phiên bản này làm cơ sở cập nhật Class Diagram trong báo cáo.</t>
+  </si>
+  <si>
+    <t>Slot 7</t>
   </si>
 </sst>
 </file>
@@ -938,4 +969,134 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD51B820-368B-424D-A8E0-DD1496A543D2}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.9375" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="3" width="28.5" customWidth="1"/>
+    <col min="4" max="4" width="54.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="13.9" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
submit audit log slot 8
</commit_message>
<xml_diff>
--- a/AI Audit Log_LeDinhThuyDuong.xlsx
+++ b/AI Audit Log_LeDinhThuyDuong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\ai-audit-log-DuongLDT2005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7BFA9A-6E47-48D0-B2F0-477A5BE5EC38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6593A408-E776-4542-9239-7ACDC1B8B9BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="67">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -118,33 +118,18 @@
     <t>“Tạo bảng phân biệt các quan hệ trong class diagram và hiệu số.”</t>
   </si>
   <si>
-    <t>Phản hồi: AI lập bảng so sánh các loại quan hệ UML, gồm association, aggregation, composition, inheritance,… và mô tả mức độ liên kết. Quyết định: Tôi nhận thấy có bổ sung quan hệ ngoài phạm vi chương nên cần tinh chỉnh theo tài liệu học.</t>
-  </si>
-  <si>
     <t>“Chỉ liệt kê những quan hệ có trong sách thôi.”</t>
   </si>
   <si>
-    <t>Phản hồi: AI giới hạn lại còn association, aggregation, composition và generalization/inheritance; đồng thời nêu các biến thể multiplicity và association types. Kiểm chứng: Tôi dùng kết quả này làm chuẩn khi ôn tập theo đúng nội dung sách thay vì UML mở rộng.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI xác định các entity classes từ yêu cầu nghiệp vụ (Customer, Booking, Vehicle, Payment, Staff, ...), xây dựng các quan hệ association, multiplicity và inheritance phù hợp rồi sinh mã PlantUML. Quyết định: Tôi sử dụng sơ đồ này làm bản nháp thiết kế trước khi tự kiểm tra lại theo nguyên tắc phân tích miền nghiệp vụ.</t>
-  </si>
-  <si>
     <t>"Tại sao service với repo thì là use?"</t>
   </si>
   <si>
-    <t>Phản hồi: AI giải thích dependency («use») biểu diễn sự phụ thuộc tạm thời giữa các lớp kỹ thuật. Quyết định: Tôi áp dụng dependency thay vì association cho Service và Repository trong design class diagram.</t>
-  </si>
-  <si>
     <t>"Dựa vào đề AutoGo thiết kế hệ thống và generate class diagram PlantUML."</t>
   </si>
   <si>
     <t>"Có thể gộp Authentication và User Management vào một Class Diagram không?"</t>
   </si>
   <si>
-    <t>Phản hồi: AI giải thích có thể gộp khi hai chức năng liên quan chặt chẽ thông qua User Entity. Quyết định: Thiết kế diagram chung cho Auth &amp; User Management.</t>
-  </si>
-  <si>
     <t>"deletedBy trong User có relationship gì không?"</t>
   </si>
   <si>
@@ -160,9 +145,6 @@
     <t>"Shared class có nên vẽ trong diagram không?"</t>
   </si>
   <si>
-    <t>Phản hồi: AI phân tích sự khác nhau giữa Feature Diagram và Architecture Diagram. Quyết định: Chỉ vẽ shared classes thực sự được sử dụng trong feature đó.</t>
-  </si>
-  <si>
     <t>"Dependency có cần bỏ trong &lt;&lt;&gt;&gt; không?"</t>
   </si>
   <si>
@@ -172,59 +154,125 @@
     <t>"Gen Class Diagram riêng cho User Management."</t>
   </si>
   <si>
-    <t>Phản hồi: AI tách User Management khỏi Authentication thành diagram độc lập. Quyết định: Áp dụng phương pháp vẽ diagram theo từng feature/module.</t>
-  </si>
-  <si>
     <t>"Phân tích class diagram Authentication Feature."</t>
   </si>
   <si>
-    <t>Phản hồi: AI phân tích vai trò của Controller, Service, Repository, Entity, Utility và các quan hệ dependency/association trong diagram. Quyết định: Tôi đối chiếu với kiến trúc ExpressJS + Mongoose của dự án để xác nhận các lớp và trách nhiệm phù hợp với implementation thực tế.</t>
-  </si>
-  <si>
     <t>"Đánh giá các relationship trong Authentication Class Diagram."</t>
   </si>
   <si>
-    <t>Phản hồi: AI giải thích dependency, association, multiplicity giữa User, RefreshToken, PasswordResetToken và Repository. Quyết định: Tôi rà soát lại các quan hệ để bảo đảm đúng ý nghĩa nghiệp vụ và thống nhất cách biểu diễn UML.</t>
-  </si>
-  <si>
     <t>"Cải thiện Authentication Class Diagram và sinh lại PlantUML."</t>
   </si>
   <si>
-    <t>Phản hồi: AI đề xuất loại bỏ các JWT methods khỏi User entity, bổ sung stereotype và điều chỉnh dependency giữa các lớp. Quyết định: Tôi cập nhật diagram theo hướng tách biệt rõ Authentication concern khỏi Entity.</t>
-  </si>
-  <si>
     <t>"Phân tích User Management Class Diagram."</t>
   </si>
   <si>
-    <t>Phản hồi: AI đánh giá trách nhiệm của UserController, UserService, UserRepository, User entity và chỉ ra các thành phần có thể không thuộc phạm vi User Management. Quyết định: Tôi điều chỉnh lại phạm vi chức năng của feature theo đúng use case quản lý người dùng.</t>
-  </si>
-  <si>
     <t>"User entity có nên chứa generateAccessToken() và generateRefreshToken() không?"</t>
   </si>
   <si>
-    <t>Phản hồi: AI giải thích việc tạo JWT thuộc Authentication concern và nên đặt ở Service hoặc Utility thay vì Entity. Quyết định: Tôi loại bỏ các JWT methods khỏi User entity để tăng tính tách biệt trách nhiệm</t>
-  </si>
-  <si>
     <t>"Sinh lại PlantUML cho User Management Feature sau khi cải thiện."</t>
   </si>
   <si>
-    <t>Phản hồi: AI tạo lại PlantUML với stereotype, dependency và association đã được chỉnh sửa. Quyết định: Tôi sử dụng phiên bản này làm cơ sở cập nhật Class Diagram trong báo cáo.</t>
-  </si>
-  <si>
     <t>Slot 7</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI lập bảng so sánh các loại quan hệ UML, gồm association, aggregation, composition, inheritance,… và mô tả mức độ liên kết.
+Quyết định: Tôi nhận thấy có bổ sung quan hệ ngoài phạm vi chương nên cần tinh chỉnh theo tài liệu học.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giới hạn lại còn association, aggregation, composition và generalization/inheritance; đồng thời nêu các biến thể multiplicity và association types.
+Kiểm chứng: Tôi dùng kết quả này làm chuẩn khi ôn tập theo đúng nội dung sách thay vì UML mở rộng.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI xác định các entity classes từ yêu cầu nghiệp vụ (Customer, Booking, Vehicle, Payment, Staff, ...), xây dựng các quan hệ association, multiplicity và inheritance phù hợp rồi sinh mã PlantUML.
+Quyết định: Tôi sử dụng sơ đồ này làm bản nháp thiết kế trước khi tự kiểm tra lại theo nguyên tắc phân tích miền nghiệp vụ.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích dependency («use») biểu diễn sự phụ thuộc tạm thời giữa các lớp kỹ thuật.
+Quyết định: Tôi áp dụng dependency thay vì association cho Service và Repository trong design class diagram.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích có thể gộp khi hai chức năng liên quan chặt chẽ thông qua User Entity.
+Quyết định: Thiết kế diagram chung cho Auth &amp; User Management.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích sự khác nhau giữa Feature Diagram và Architecture Diagram.
+Quyết định: Chỉ vẽ shared classes thực sự được sử dụng trong feature đó.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI tách User Management khỏi Authentication thành diagram độc lập.
+Quyết định: Áp dụng phương pháp vẽ diagram theo từng feature/module.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích vai trò của Controller, Service, Repository, Entity, Utility và các quan hệ dependency/association trong diagram.
+Quyết định: Tôi đối chiếu với kiến trúc ExpressJS + Mongoose của dự án để xác nhận các lớp và trách nhiệm phù hợp với implementation thực tế.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích dependency, association, multiplicity giữa User, RefreshToken, PasswordResetToken và Repository.
+Quyết định: Tôi rà soát lại các quan hệ để bảo đảm đúng ý nghĩa nghiệp vụ và thống nhất cách biểu diễn UML.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất loại bỏ các JWT methods khỏi User entity, bổ sung stereotype và điều chỉnh dependency giữa các lớp.
+Quyết định: Tôi cập nhật diagram theo hướng tách biệt rõ Authentication concern khỏi Entity.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đánh giá trách nhiệm của UserController, UserService, UserRepository, User entity và chỉ ra các thành phần có thể không thuộc phạm vi User Management.
+Quyết định: Tôi điều chỉnh lại phạm vi chức năng của feature theo đúng use case quản lý người dùng.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích việc tạo JWT thuộc Authentication concern và nên đặt ở Service hoặc Utility thay vì Entity.
+Quyết định: Tôi loại bỏ các JWT methods khỏi User entity để tăng tính tách biệt trách nhiệm</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI tạo lại PlantUML với stereotype, dependency và association đã được chỉnh sửa.
+Quyết định: Tôi sử dụng phiên bản này làm cơ sở cập nhật Class Diagram trong báo cáo.</t>
+  </si>
+  <si>
+    <t>"Gen sequence diagram khi có class như trong class diagram cho UC Login, tham khảo các quy tắc vẽ tại Một số lưu ý."</t>
+  </si>
+  <si>
+    <t>"Nếu có API Gateway vào giữa thì sao?"</t>
+  </si>
+  <si>
+    <t>"Như structure StallBox hiện tại có API Gateway không?"</t>
+  </si>
+  <si>
+    <t>Slot 8</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI sinh sequence diagram cho UC Login dựa trên kiến trúc Controller – Service – Repository – Entity và các quy tắc UML được cung cấp.
+Quyết định: Tôi đối chiếu với source code và kiến trúc dự án StallBox để điều chỉnh participant và message cho phù hợp với thực tế triển khai.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI xác định vai trò của Controller, Service, Repository, Entity và Utility.
+Quyết định: Tôi dùng kết quả này để xác định các participant cần xuất hiện trong sequence diagram Login.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI mô tả cách bổ sung API Gateway vào sequence diagram và ảnh hưởng của nó tới luồng giao tiếp giữa Frontend và Backend.
+Quyết định: Tôi xem xét khả năng mở rộng kiến trúc trong tương lai nhưng chưa áp dụng cho thiết kế hiện tại.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích cấu trúc dự án và xác định hệ thống chưa sử dụng API Gateway riêng biệt.
+Quyết định: Tôi giữ mô hình giao tiếp trực tiếp giữa client và backend trong sequence diagram.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -278,12 +326,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -294,6 +342,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -766,7 +817,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -825,7 +876,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -836,7 +887,7 @@
         <v>26</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
@@ -847,10 +898,10 @@
         <v>22</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="81" x14ac:dyDescent="0.35">
@@ -861,10 +912,10 @@
         <v>22</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="54" x14ac:dyDescent="0.35">
@@ -875,13 +926,13 @@
         <v>22</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="54" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -889,10 +940,10 @@
         <v>22</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="27" x14ac:dyDescent="0.35">
@@ -903,10 +954,10 @@
         <v>22</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="54" x14ac:dyDescent="0.35">
@@ -917,13 +968,13 @@
         <v>22</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="54" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -931,10 +982,10 @@
         <v>22</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
@@ -945,13 +996,13 @@
         <v>22</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="54" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -959,21 +1010,21 @@
         <v>22</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD51B820-368B-424D-A8E0-DD1496A543D2}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.9375" customWidth="1"/>
@@ -997,18 +1048,18 @@
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="81" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="54" x14ac:dyDescent="0.35">
@@ -1016,13 +1067,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="54" x14ac:dyDescent="0.35">
@@ -1030,13 +1081,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
@@ -1044,13 +1095,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
@@ -1058,13 +1109,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="54" x14ac:dyDescent="0.35">
@@ -1072,31 +1123,87 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="40.5" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="54" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>57</v>
+    </row>
+    <row r="9" spans="1:5" ht="81" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
submit ai audit log week 5
</commit_message>
<xml_diff>
--- a/AI Audit Log_LeDinhThuyDuong.xlsx
+++ b/AI Audit Log_LeDinhThuyDuong.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\ai-audit-log-DuongLDT2005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6593A408-E776-4542-9239-7ACDC1B8B9BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5677081E-1BCA-4673-9412-F727390E20BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
     <sheet name="Week 3" sheetId="5" r:id="rId2"/>
     <sheet name="Week 4" sheetId="6" r:id="rId3"/>
+    <sheet name="Week 5" sheetId="8" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="85">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -253,19 +254,88 @@
   <si>
     <t>Phản hồi: AI phân tích cấu trúc dự án và xác định hệ thống chưa sử dụng API Gateway riêng biệt.
 Quyết định: Tôi giữ mô hình giao tiếp trực tiếp giữa client và backend trong sequence diagram.</t>
+  </si>
+  <si>
+    <t>"Thiết kế Sequence Diagram theo Layered Architecture cho Use Case Create Booking and Pay Deposit."</t>
+  </si>
+  <si>
+    <t>"Bổ sung Repository Pattern vào Sequence Diagram."</t>
+  </si>
+  <si>
+    <t>"Kiểm tra điều kiện Car Availability trong Sequence Diagram."</t>
+  </si>
+  <si>
+    <t>"Mô hình hóa Payment Success và Payment Failure trong Sequence Diagram."</t>
+  </si>
+  <si>
+    <t>"Sinh PlantUML Sequence Diagram từ mô tả nghiệp vụ."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI tạo mã PlantUML hoàn chỉnh thể hiện đầy đủ lifeline, activation, repository calls, điều kiện kiểm tra xe và thanh toán. Quyết định: Tôi sử dụng mã PlantUML làm bản nháp ban đầu, sau đó chỉnh sửa lại bố cục và tên phương thức cho phù hợp với thiết kế cuối cùng.</t>
+  </si>
+  <si>
+    <t>"Đối chiếu Sequence Diagram với Class Diagram và kiến trúc hệ thống."</t>
+  </si>
+  <si>
+    <t>"Đánh giá Sequence Diagram theo hướng dẫn Report và UML Best Practices."</t>
+  </si>
+  <si>
+    <t>"Phân tích source code/backend flow để sinh Sequence Diagram chi tiết."</t>
+  </si>
+  <si>
+    <t>Slot 9</t>
+  </si>
+  <si>
+    <t>Slot 10</t>
+  </si>
+  <si>
+    <t>theo Layered Architecture cho Use Case Create Booking and Pay Deposit."
+Phản hồi: AI đề xuất luồng tương tác từ Actor → Boundary → Controller → Service → Repository → Entity, bảo đảm đúng nguyên tắc phân tầng và tách biệt trách nhiệm.
+Quyết định: Tôi áp dụng cấu trúc phân tầng này để thống nhất với kiến trúc hệ thống được lựa chọn trong bài thi.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất các lời gọi phương thức như findAvailableCar(), createBooking(), saveBooking(), processDeposit() thông qua Repository thay vì truy cập trực tiếp dữ liệu. 
+Quyết định: Tôi cập nhật Sequence Diagram để thể hiện rõ Repository Pattern theo yêu cầu đề bài.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất sử dụng Combined Fragment «alt» với hai nhánh: Car Available và Car Not Available. Nếu xe không khả dụng, hệ thống trả thông báo lỗi và kết thúc luồng.
+Quyết định: Tôi bổ sung alt fragment để mô hình hóa đúng luồng nghiệp vụ và đáp ứng yêu cầu UML.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất alt fragment thứ hai cho kết quả thanh toán. Nếu thanh toán thành công thì xác nhận booking; nếu thất bại thì hủy booking và cập nhật trạng thái tương ứng.
+Quyết định: Tôi bổ sung hai nhánh xử lý để phản ánh đầy đủ nghiệp vụ thanh toán đặt cọc.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI kiểm tra sự nhất quán giữa các lớp Service, Repository, Entity xuất hiện trong Class Diagram với các lifeline trong Sequence Diagram.
+Quyết định: Tôi điều chỉnh lại tên lớp và lời gọi phương thức để bảo đảm traceability giữa các UML artifacts.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất sử dụng Boundary–Control–Entity, hạn chế Actor gọi trực tiếp Repository hoặc Entity, đồng thời duy trì luồng tương tác rõ ràng từ giao diện đến cơ sở dữ liệu.
+Quyết định: Tôi chuẩn hóa diagram theo mô hình BCE nhằm tăng tính dễ hiểu và tuân thủ hướng dẫn môn học.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI truy vết luồng xử lý từ API Request đến Controller, Service, Repository và Database, đồng thời đề xuất các message tương ứng cho từng bước xử lý.
+Quyết định: Tôi sử dụng kết quả phân tích này để xây dựng Sequence Diagram sát với implementation thực tế thay vì chỉ mô tả nghiệp vụ ở mức khái niệm.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -326,12 +396,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -342,6 +412,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -817,7 +890,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1017,7 +1090,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1203,7 +1276,151 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C588554B-D1EB-4D8A-A3D1-794E377F2705}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.9375" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="3" width="28.5" customWidth="1"/>
+    <col min="4" max="4" width="54.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="13.9" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="94.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="81" x14ac:dyDescent="0.35">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="81" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
submit audit log week 7
</commit_message>
<xml_diff>
--- a/AI Audit Log_LeDinhThuyDuong.xlsx
+++ b/AI Audit Log_LeDinhThuyDuong.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\ai-audit-log-DuongLDT2005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5677081E-1BCA-4673-9412-F727390E20BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C12BA4BF-D549-4011-8CEE-F6E3B289C106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="5" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
     <sheet name="Week 3" sheetId="5" r:id="rId2"/>
     <sheet name="Week 4" sheetId="6" r:id="rId3"/>
     <sheet name="Week 5" sheetId="8" r:id="rId4"/>
+    <sheet name="Week 6" sheetId="9" r:id="rId5"/>
+    <sheet name="Week 7" sheetId="10" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="119">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -316,19 +318,142 @@
   <si>
     <t>Phản hồi: AI truy vết luồng xử lý từ API Request đến Controller, Service, Repository và Database, đồng thời đề xuất các message tương ứng cho từng bước xử lý.
 Quyết định: Tôi sử dụng kết quả phân tích này để xây dựng Sequence Diagram sát với implementation thực tế thay vì chỉ mô tả nghiệp vụ ở mức khái niệm.</t>
+  </si>
+  <si>
+    <t>"Thiết kế Activity Diagram Return Car theo Swimlane."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI xác định các swimlane gồm Staff và System, đồng thời đề xuất luồng kiểm tra xe, tính phí phát sinh và hoàn tất booking.
+Quyết định: Tôi sử dụng mô hình Swimlane Level 2 (Design Level) theo đúng yêu cầu đề bài.</t>
+  </si>
+  <si>
+    <t>"Giải thích Merge Node và Decision Node trong Activity Diagram."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích vai trò của Decision Node trong việc phân nhánh và Merge Node trong việc hợp nhất các luồng xử lý. 
+Quyết định: Tôi chỉnh sửa Activity Diagram để sử dụng đúng ký hiệu UML chuẩn.</t>
+  </si>
+  <si>
+    <t>"Xác định các Activity và Action trong Use Case Return Car."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích các bước nghiệp vụ gồm nhận xe, kiểm tra tình trạng xe, xác định phí phát sinh, cập nhật trạng thái booking và hoàn tất giao dịch.
+Quyết định: Tôi sử dụng các action này làm cơ sở xây dựng Activity Diagram.</t>
+  </si>
+  <si>
+    <t>"Thiết kế luồng xử lý Additional Fee trong Activity Diagram."</t>
+  </si>
+  <si>
+    <t>"Kiểm tra tính đúng đắn của Activity Diagram theo chuẩn UML."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI rà soát Start Node, Activity Flow, Decision Node, Merge Node và End Node, đồng thời đề xuất chỉnh sửa các luồng chưa hợp lệ. 
+Quyết định: Tôi cập nhật sơ đồ để tuân thủ ký pháp UML chuẩn.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất sử dụng Decision Node để xác định xe có hư hỏng hay phát sinh phí bổ sung hay không, sau đó chuyển sang các nhánh xử lý tương ứng. 
+Quyết định: Tôi bổ sung nhánh điều kiện để mô hình hóa nghiệp vụ đầy đủ hơn.</t>
+  </si>
+  <si>
+    <t>"Xác định các trạng thái của Booking trong State Diagram."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất các trạng thái Draft, Pending Payment, Confirmed, Active Rental, Returned, Completed và Cancelled phản ánh toàn bộ vòng đời booking.
+Quyết định: Tôi sử dụng các trạng thái này để xây dựng State Diagram cho thực thể Booking.</t>
+  </si>
+  <si>
+    <t>"Mô hình hóa trạng thái khi khách hàng trả xe."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất chuyển trạng thái từ Active Rental sang Returned, sau đó sang Completed sau khi xử lý các khoản phí phát sinh. 
+Quyết định: Tôi bổ sung các transition này để thể hiện đầy đủ vòng đời thuê xe.</t>
+  </si>
+  <si>
+    <t>"Kiểm tra State Diagram giữa Booking và Vehicle."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích mối liên hệ giữa trạng thái Booking và Vehicle nhằm bảo đảm tính đồng bộ trong nghiệp vụ thuê xe. Quyết định: Tôi điều chỉnh các trạng thái để tránh xung đột và phản ánh đúng quy trình thực tế.</t>
+  </si>
+  <si>
+    <t>Slot 11</t>
+  </si>
+  <si>
+    <t>Slot 12</t>
+  </si>
+  <si>
+    <t>"Thiết kế Component Diagram cho AutoGo theo Layered Architecture."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất các tầng Presentation Layer, Business Layer, Repository Layer và Database Layer cùng các dependency giữa các tầng.
+Quyết định: Tôi sử dụng cấu trúc này để xây dựng Component Diagram thống nhất với các diagram trước đó.</t>
+  </si>
+  <si>
+    <t>"Phân tích các component cần có trong AutoGo theo Layered Architecture."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất chia hệ thống thành Presentation Layer, Business Layer, Repository Layer và Database Layer, đồng thời xác định các service chính gồm UserService, VehicleService, BookingService và PaymentService. 
+Quyết định: Tôi sử dụng cấu trúc này làm nền tảng cho Component Diagram.</t>
+  </si>
+  <si>
+    <t>"Xác định interface và dependency giữa các component."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất mỗi service chỉ giao tiếp với repository tương ứng thông qua interface nhằm giảm coupling và tăng khả năng mở rộng. 
+Quyết định: Tôi áp dụng dependency thông qua interface repository thay vì phụ thuộc trực tiếp vào implementation.</t>
+  </si>
+  <si>
+    <t>"Kiểm tra Component Diagram có vi phạm nguyên tắc Layered Architecture hay không."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phát hiện một số dependency bỏ qua tầng Repository và truy cập trực tiếp Database Layer, đồng thời đề xuất chỉnh sửa để bảo đảm nguyên tắc phân tầng.
+Quyết định: Tôi cập nhật lại các dependency giữa các component.</t>
+  </si>
+  <si>
+    <t>Slot 13</t>
+  </si>
+  <si>
+    <t>Slot 14</t>
+  </si>
+  <si>
+    <t>"Xác định đối tượng phù hợp để xây dựng State Diagram."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích các thực thể trong hệ thống và đề xuất Booking là đối tượng có vòng đời rõ ràng nhất, phù hợp để mô hình hóa bằng State Diagram.
+Quyết định: Tôi chọn Booking làm đối tượng chính cho State Diagram.</t>
+  </si>
+  <si>
+    <t>"Liệt kê các trạng thái trong vòng đời của Booking."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất các trạng thái Pending, Confirmed, Active, Returned, Completed và Cancelled theo đúng quy trình thuê xe.
+Quyết định: Tôi sử dụng các trạng thái này làm cơ sở xây dựng State Diagram.</t>
+  </si>
+  <si>
+    <t>"Kiểm tra tính hợp lệ của các transition trong State Diagram."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phát hiện một số transition chưa hợp lý, chẳng hạn chuyển trực tiếp từ Pending sang Completed mà bỏ qua các trạng thái trung gian.
+Quyết định: Tôi điều chỉnh lại các transition để phản ánh đúng nghiệp vụ.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -396,12 +521,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -412,6 +537,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -890,7 +1018,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1090,7 +1218,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1276,7 +1404,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1420,7 +1548,281 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E412E75A-0C37-488F-80A1-0058DD7EAB5B}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.9375" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="3" width="28.5" customWidth="1"/>
+    <col min="4" max="4" width="54.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="13.9" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{238EA005-EF30-4717-86D9-913B10D99926}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.9375" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="3" width="28.5" customWidth="1"/>
+    <col min="4" max="4" width="54.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="13.9" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="81" x14ac:dyDescent="0.35">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="54" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="67.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>